<commit_message>
feat(F-NAR-019): ATOM-AUT.RAN.001-02 Le cacao de Nina
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.RAN.001-02.xlsx
+++ b/stories/arbres/ATOM-AUT.RAN.001-02.xlsx
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nina veut le vrai cacao sur le tapis, avec son ours. L'ours disparaît sous le pique-nique. Elle met tasses et peluches dans la caisse pour chercher. L'ours apparaît sous la poule. Ils boivent.</t>
+          <t>Nina veut le cacao au milieu du tapis, maintenant, pour son ours. Une lune d'étain brille sur la boîte à musique. L'ours disparaît sous le pique-nique. Elle cherche le lit, pousse le tas : rien. Elle refuse de foncer, pose les tasses dans la caisse, suit la lune, trouve l'ours sous la poule. La vapeur du cacao s'accroche à la lune d'étain.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Trois notes sortent de la boîte à musique. Ding. Puis plus rien. Une chaussette sèche sur la chaise. Elle est encore un peu tiède. Dehors, les feuilles sont mouillées. Il fait frais, ce soir. Le cacao est sur le feu. Dans la chambre, le tapis est épais. Un ours en peluche attend sur l'oreiller. Il est tout doux, un peu chaud. En ce moment, Nina est à genoux. Elle prend l'ours contre sa joue. Toi, tu viens au tapis. Un lapin et une poule attendent déjà. Nina pose trois tasses en bois. Les tasses font clic. C'est un pique-nique ! Un pique-nique pour les peluches. Nina donne une tasse à l'ours. Elle donne une tasse au lapin. La poule a la petite tasse. Ils sont bien installés. Ils boivent du cacao, papa. Du cacao en bois, alors. Nina souffle au-dessus d'une tasse. Ffff. Le vrai cacao arrive bientôt. On le boit ici, sur le tapis ? Oui, au milieu, tout chaud. Maman entre avec la grande tasse. Ça sent le cacao, tout près. Une petite vapeur monte. Nina cherche un rond pour la tasse. Une tasse en bois est déjà là. La patte du lapin est dessus. L'ours veut le vrai cacao aussi. Où est-il, ton ours ? Nina regarde l'oreiller. L'oreiller est plat, vide. Il n'est plus sur le lit. Sous la couverture ? Elle soulève la couverture rose. Rien, seulement le drap tiède. Il est perdu. Les peluches et les tasses couvrent le tapis. Je n'ai pas de place. Il faut un petit rond, au milieu. Nina prend une tasse en bois. Elle la pose dans la caisse ronde. Clic. Je cherche dessous.</t>
+          <t>La vapeur du cacao grimpe l'escalier. Elle entre dans la chambre froide. Sur la vitre, la pluie trace un chemin. La boîte à musique vient de se taire. Un ding reste coincé dans l'air. Sur le couvercle, une lune d'étain. Elle capte un bout de ciel gris. La lumière est basse, un peu bleue. Une chaussette sèche sur la chaise. Elle est un peu tiède. La chambre sent le cacao chaud. Il fait frais, ce soir. Le cacao est sur le feu. Je le veux sur le tapis ! Maintenant, maman. Il va refroidir vite. En ce moment, Nina s'agenouille. Le tapis est épais, un peu froid. Un ours brun attend sur l'oreiller. Toi, tu viens au pique-nique. Elle le pose au milieu du tapis. Un lapin gris la rejoint. Une poule jaune s'installe près de lui. Nina aligne trois tasses en bois. Les tasses font clic. C'est pour le vrai cacao. Il arrive, bien chaud. Vous soufflerez dessus. Nina souffle au-dessus d'une tasse. Ffff. Maman pousse la porte, une grande tasse à la main. Une petite vapeur danse au bord. Pose-la au milieu ! Nina cherche un rond libre. La patte du lapin occupe le centre. L'ours veut le cacao, lui. Où est ton ours, alors ? Nina se tourne vers l'oreiller. L'oreiller est plat, vide. Il n'est plus sur le lit. Sous la couverture rose ? Elle soulève la couverture. Rien, seulement le drap tiède. Il est perdu ! Le sourire de Nina disparaît. Les peluches et les tasses couvrent le tapis. Je n'ai pas de place. Nina pousse le tas d'un bras. Une tasse roule vers la chaise. Le tas retombe, plus mêlé. Ça ne marche pas. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Maman s'accroupit à la même hauteur. Tu veux pousser, ou regarder ? Je veux mon ours. Nina baisse les épaules.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Trois notes sortent de la boîte à musique. Ding. Puis plus rien. Une chaussette sèche sur la chaise. Elle est encore un peu tiède. Dehors, les feuilles sont mouillées. Il fait frais, ce soir. Le cacao est sur le feu. Dans la chambre, le tapis est épais. Un ours en peluche attend sur l'oreiller. Il est tout doux, un peu chaud. En ce moment, Nina est à genoux. Elle prend l'ours contre sa joue. Toi, tu viens au tapis. Un lapin et une poule attendent déjà. Nina pose trois tasses en bois. Les tasses font clic. C'est un pique-nique ! Un pique-nique pour les peluches. Nina donne une tasse à l'ours. Elle donne une tasse au lapin. La poule a la petite tasse. Ils sont bien installés. Ils boivent du cacao, papa. Du cacao en bois, alors. Nina souffle au-dessus d'une tasse. Ffff. Le vrai cacao arrive bientôt. On le boit ici, sur le tapis ? Oui, au milieu, tout chaud. Maman entre avec la grande tasse. Ça sent le cacao, tout près. Une petite vapeur monte. Nina cherche un rond pour la tasse. Une tasse en bois est déjà là. La patte du lapin est dessus. L'ours veut le vrai cacao aussi. Où est-il, ton ours ? Nina regarde l'oreiller. L'oreiller est plat, vide. Il n'est plus sur le lit. Sous la couverture ? Elle soulève la couverture rose. Rien, seulement le drap tiède. Il est perdu. Les peluches et les tasses couvrent le tapis. Je n'ai pas de place. Il faut un petit rond, au milieu. Nina prend une tasse en bois. Elle la pose dans la caisse ronde. Clic. Je cherche dessous.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La vapeur du cacao grimpe l'escalier. Elle entre dans la chambre froide. Sur la vitre, la pluie trace un chemin. La boîte à musique vient de se taire. Un ding reste coincé dans l'air. Sur le couvercle, une &lt;emphasis level="moderate"&gt;lune d'étain&lt;/emphasis&gt;. Elle capte un bout de ciel gris. La lumière est basse, un peu bleue. Une chaussette sèche sur la chaise. Elle est un peu tiède. La chambre sent le cacao chaud. Il fait frais, ce soir. Le cacao est sur le feu. Je le veux sur le tapis ! Maintenant, maman. Il va refroidir vite. En ce moment, Nina s'agenouille. Le tapis est épais, un peu froid. Un ours brun attend sur l'oreiller. Toi, tu viens au pique-nique. Elle le pose au milieu du tapis. Un lapin gris la rejoint. Une poule jaune s'installe près de lui. Nina aligne trois tasses en bois. Les tasses font clic. C'est pour le vrai cacao. Il arrive, bien chaud. Vous soufflerez dessus. Nina souffle au-dessus d'une tasse. Ffff. Maman pousse la porte, une grande tasse à la main. Une petite vapeur danse au bord. Pose-la au milieu ! Nina cherche un rond libre. La patte du lapin occupe le centre. L'ours veut le cacao, lui. Où est ton ours, alors ? Nina se tourne vers l'oreiller. L'oreiller est plat, vide. Il n'est plus sur le lit. Sous la couverture rose ? Elle soulève la couverture. Rien, seulement le drap tiède. Il est perdu ! Le sourire de Nina disparaît. Les peluches et les tasses couvrent le tapis. Je n'ai pas de place. Nina pousse le tas d'un bras. Une tasse roule vers la chaise. Le tas retombe, plus mêlé. Ça ne marche pas. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Maman s'accroupit à la même hauteur. Tu veux pousser, ou regarder ? Je veux mon ours. Nina baisse les épaules.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Sami joue dans sa chambre. Maman plie des chaussettes. Sami a des peluches. Les peluches sont douces. Sami fait un pique-nique. Les tasses en bois font clic. Puis le jeu est fini. Maman dit : c'est l'heure de &lt;emphasis&gt;ranger&lt;/emphasis&gt;. Ranger, c'est mettre dans la caisse. Sami prend une peluche. Il la met dans la caisse. Il prend un livre. Il le met dans la caisse. Encore une peluche. Dans la caisse. La caisse est pleine. Le tapis est vide. Parce qu'il range, la chambre est calme. Maman dit : merci Sami. Sami ferme le couvercle. Ça fait toc. [pause]</t>
+          <t>La vapeur du cacao grimpe l'escalier. Elle entre dans la chambre froide. Sur la vitre, la pluie trace un chemin. La boîte à musique vient de se taire. Un ding reste coincé dans l'air. Sur le couvercle, une &lt;emphasis&gt;lune d'étain&lt;/emphasis&gt;. Elle capte un bout de ciel gris. La lumière est basse, un peu bleue. Une chaussette sèche sur la chaise. Elle est un peu tiède. La chambre sent le cacao chaud. Il fait frais, ce soir. Le cacao est sur le feu. Je le veux sur le tapis ! Maintenant, maman. Il va refroidir vite. En ce moment, Nina s'agenouille. Le tapis est épais, un peu froid. Un ours brun attend sur l'oreiller. Toi, tu viens au pique-nique. Elle le pose au milieu du tapis. Un lapin gris la rejoint. Une poule jaune s'installe près de lui. Nina aligne trois tasses en bois. Les tasses font clic. C'est pour le vrai cacao. Il arrive, bien chaud. Vous soufflerez dessus. Nina souffle au-dessus d'une tasse. Ffff. Maman pousse la porte, une grande tasse à la main. Une petite vapeur danse au bord. Pose-la au milieu ! Nina cherche un rond libre. La patte du lapin occupe le centre. L'ours veut le cacao, lui. Où est ton ours, alors ? Nina se tourne vers l'oreiller. L'oreiller est plat, vide. Il n'est plus sur le lit. Sous la couverture rose ? Elle soulève la couverture. Rien, seulement le drap tiède. Il est perdu ! Le sourire de Nina disparaît. Les peluches et les tasses couvrent le tapis. Je n'ai pas de place. Nina pousse le tas d'un bras. Une tasse roule vers la chaise. Le tas retombe, plus mêlé. Ça ne marche pas. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Maman s'accroupit à la même hauteur. Tu veux pousser, ou regarder ? Je veux mon ours. Nina baisse les épaules. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>ranger</t>
+          <t>lune d'étain</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,61 +1321,75 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller; emotion=impatience_curieuse; intensite=2; destinataire=enfant; sous_texte=la_lune_detain_sur_la_boite; tempo=naturel; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Trois notes sortent de la boîte à musique.
-narrateur|Ding.
-narrateur|Puis plus rien.
+          <t>narrateur|La vapeur du cacao grimpe l'escalier.
+narrateur|Elle entre dans la chambre froide.
+narrateur|Sur la vitre, la pluie trace un chemin.
+narrateur|La boîte à musique vient de se taire.
+narrateur|Un ding reste coincé dans l'air.
+narrateur|Sur le couvercle, une lune d'étain.
+narrateur|Elle capte un bout de ciel gris.
+narrateur|La lumière est basse, un peu bleue.
 narrateur|Une chaussette sèche sur la chaise.
-narrateur|Elle est encore un peu tiède.
-narrateur|Dehors, les feuilles sont mouillées.
+narrateur|Elle est un peu tiède.
+narrateur|La chambre sent le cacao chaud.
 papa|Il fait frais, ce soir.
 maman|Le cacao est sur le feu.
-narrateur|Dans la chambre, le tapis est épais.
-narrateur|Un ours en peluche attend sur l'oreiller.
-narrateur|Il est tout doux, un peu chaud.
-narrateur|En ce moment, Nina est à genoux.
-narrateur|Elle prend l'ours contre sa joue.
-enfant-f|Toi, tu viens au tapis.
-narrateur|Un lapin et une poule attendent déjà.
-narrateur|Nina pose trois tasses en bois.
+enfant-f|Je le veux sur le tapis !
+enfant-f|Maintenant, maman.
+maman|Il va refroidir vite.
+narrateur|En ce moment, Nina s'agenouille.
+narrateur|Le tapis est épais, un peu froid.
+narrateur|Un ours brun attend sur l'oreiller.
+enfant-f|Toi, tu viens au pique-nique.
+narrateur|Elle le pose au milieu du tapis.
+narrateur|Un lapin gris la rejoint.
+narrateur|Une poule jaune s'installe près de lui.
+narrateur|Nina aligne trois tasses en bois.
 narrateur|Les tasses font clic.
-enfant-f|C'est un pique-nique !
-maman|Un pique-nique pour les peluches.
-narrateur|Nina donne une tasse à l'ours.
-narrateur|Elle donne une tasse au lapin.
-narrateur|La poule a la petite tasse.
-papa|Ils sont bien installés.
-enfant-f|Ils boivent du cacao, papa.
-papa|Du cacao en bois, alors.
+enfant-f|C'est pour le vrai cacao.
+maman|Il arrive, bien chaud.
+papa|Vous soufflerez dessus.
 narrateur|Nina souffle au-dessus d'une tasse.
 enfant-f|Ffff.
-maman|Le vrai cacao arrive bientôt.
-enfant-f|On le boit ici, sur le tapis ?
-maman|Oui, au milieu, tout chaud.
-narrateur|Maman entre avec la grande tasse.
-narrateur|Ça sent le cacao, tout près.
-narrateur|Une petite vapeur monte.
-narrateur|Nina cherche un rond pour la tasse.
-narrateur|Une tasse en bois est déjà là.
-narrateur|La patte du lapin est dessus.
-enfant-f|L'ours veut le vrai cacao aussi.
-maman|Où est-il, ton ours ?
-narrateur|Nina regarde l'oreiller.
+narrateur|Maman pousse la porte, une grande tasse à la main.
+narrateur|Une petite vapeur danse au bord.
+enfant-f|Pose-la au milieu !
+narrateur|Nina cherche un rond libre.
+narrateur|La patte du lapin occupe le centre.
+enfant-f|L'ours veut le cacao, lui.
+maman|Où est ton ours, alors ?
+narrateur|Nina se tourne vers l'oreiller.
 narrateur|L'oreiller est plat, vide.
 enfant-f|Il n'est plus sur le lit.
-papa|Sous la couverture ?
-narrateur|Elle soulève la couverture rose.
+papa|Sous la couverture rose ?
+narrateur|Elle soulève la couverture.
 narrateur|Rien, seulement le drap tiède.
-enfant-f|Il est perdu.
+enfant-f|Il est perdu !
+narrateur|Le sourire de Nina disparaît.
 narrateur|Les peluches et les tasses couvrent le tapis.
 enfant-f|Je n'ai pas de place.
-maman|Il faut un petit rond, au milieu.
-narrateur|Nina prend une tasse en bois.
-narrateur|Elle la pose dans la caisse ronde.
-narrateur|Clic.
-enfant-f|Je cherche dessous.</t>
+narrateur|Nina pousse le tas d'un bras.
+narrateur|Une tasse roule vers la chaise.
+narrateur|Le tas retombe, plus mêlé.
+enfant-f|Ça ne marche pas.
+narrateur|Dans sa poitrine, ça se bouscule.
+narrateur|L'envie et l'inquiétude se heurtent.
+narrateur|Maman s'accroupit à la même hauteur.
+maman|Tu veux pousser, ou regarder ?
+enfant-f|Je veux mon ours.
+narrateur|Nina baisse les épaules.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>pluie,boite-musique</t>
         </is>
       </c>
     </row>
@@ -1402,17 +1416,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Nina cherche son ours. Où est-il ?</t>
+          <t>Nina cherche son ours sous le tas. Où se cache-t-il ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Nina cherche son ours. Où est-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nina cherche son &lt;emphasis level="moderate"&gt;ours&lt;/emphasis&gt; sous le tas. Où se cache-t-il ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Après le jeu, que fait Sami ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nina cherche son &lt;emphasis&gt;ours&lt;/emphasis&gt; sous le tas. Où se cache-t-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1475,7 +1489,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1486,7 +1500,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1501,34 +1515,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>ours</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1543,23 +1561,23 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=l_ours_est_sous_le_tas; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Nina cherche son ours.
-narrateur|Où est-il ?</t>
+          <t>narrateur|Nina cherche son ours sous le tas.
+maman|Où se cache-t-il ?</t>
         </is>
       </c>
     </row>
@@ -1586,17 +1604,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>La deuxième tasse va dans la caisse. Clic. Nina prend le lapin tout doux. Elle le glisse dans la caisse. Tu regardes bien sous les peluches ? Oui, maman. La poule est encore au milieu. Un coin de tapis reparaît. Nina soulève la poule. Un museau brun est dessous. Mon ours ! L'ours était sous la poule. Une tasse en bois l'avait caché. Nina le serre contre sa joue. Le poil est chaud, un peu écrasé. Merci, tu l'as trouvé. Il buvait en dessous. Te voilà, petit ours. La dernière tasse va dans la caisse. Le tapis a un rond vide, au milieu. Nina pose l'ours contre son genou.</t>
+          <t>J'arrête de pousser. Elle lâche le tas. Près de la fenêtre, la lune d'étain brille. Elle me montre le tapis. Nina prend une tasse en bois. Elle la pose dans la caisse ronde. Clic. La tasse a sa place. La deuxième tasse suit. Toi aussi, lapin. Elle glisse le lapin dans la caisse. Tu regardes bien dessous ? Oui, maman. Un coin de tapis reparaît. La poule reste au milieu. Je prends tout d'un coup. Nina ouvre les deux mains. Elle veut vider le tapis vite. La poule bascule sur le côté. Puis la dernière tasse part sous la chaise. Oh non. Nina s'arrête net. Pas comme ça. Elle refuse de foncer. Elle lève les yeux vers la boîte. La lune d'étain capte la pluie. Un reflet tombe sur un petit dos. Là, sous la poule. Nina soulève la poule, sans se presser. Un museau brun est dessous. Mon ours ! L'ours était sous la poule. Une tasse en bois l'avait caché. Nina le serre contre sa joue. Le poil est chaud, un peu écrasé. Merci d'avoir regardé, Nina. Il buvait en dessous. Te voilà, petit ours. La dernière tasse va dans la caisse. Le tapis a un rond vide, au milieu. Nina pose l'ours contre son genou.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>La deuxième tasse va dans la caisse. Clic. Nina prend le lapin tout doux. Elle le glisse dans la caisse. Tu regardes bien sous les peluches ? Oui, maman. La poule est encore au milieu. Un coin de tapis reparaît. Nina soulève la poule. Un museau brun est dessous. Mon ours ! L'ours était sous la poule. Une tasse en bois l'avait caché. Nina le serre contre sa joue. Le poil est chaud, un peu écrasé. Merci, tu l'as trouvé. Il buvait en dessous. Te voilà, petit ours. La dernière tasse va dans la caisse. Le tapis a un rond vide, au milieu. Nina pose l'ours contre son genou.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;J'arrête de pousser. Elle lâche le tas. Près de la fenêtre, la &lt;emphasis level="moderate"&gt;lune d'étain&lt;/emphasis&gt; brille. Elle me montre le tapis. Nina prend une tasse en bois. Elle la pose dans la caisse ronde. Clic. La tasse a sa place. La deuxième tasse suit. Toi aussi, lapin. Elle glisse le lapin dans la caisse. Tu regardes bien dessous ? Oui, maman. Un coin de tapis reparaît. La poule reste au milieu. Je prends tout d'un coup. Nina ouvre les deux mains. Elle veut vider le tapis vite. La poule bascule sur le côté. Puis la dernière tasse part sous la chaise. Oh non. Nina s'arrête net. Pas comme ça. Elle refuse de foncer. Elle lève les yeux vers la boîte. La lune d'étain capte la pluie. Un reflet tombe sur un petit dos. Là, sous la poule. Nina soulève la poule, sans se presser. Un museau brun est dessous. Mon ours ! L'ours était sous la poule. Une tasse en bois l'avait caché. Nina le serre contre sa joue. Le poil est chaud, un peu écrasé. Merci d'avoir regardé, Nina. Il buvait en dessous. Te voilà, petit ours. La dernière tasse va dans la caisse. Le tapis a un rond vide, au milieu. Nina pose l'ours contre son genou.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Sami a rangé. Les peluches sont dans la &lt;emphasis&gt;caisse&lt;/emphasis&gt;. Le tapis est libre. Maman est là. [pause]</t>
+          <t>J'arrête de pousser. Elle lâche le tas. Près de la fenêtre, la &lt;emphasis&gt;lune d'étain&lt;/emphasis&gt; brille. Elle me montre le tapis. Nina prend une tasse en bois. Elle la pose dans la caisse ronde. Clic. La tasse a sa place. La deuxième tasse suit. Toi aussi, lapin. Elle glisse le lapin dans la caisse. Tu regardes bien dessous ? Oui, maman. Un coin de tapis reparaît. La poule reste au milieu. Je prends tout d'un coup. Nina ouvre les deux mains. Elle veut vider le tapis vite. La poule bascule sur le côté. Puis la dernière tasse part sous la chaise. Oh non. Nina s'arrête net. Pas comme ça. Elle refuse de foncer. Elle lève les yeux vers la boîte. La lune d'étain capte la pluie. Un reflet tombe sur un petit dos. Là, sous la poule. Nina soulève la poule, sans se presser. Un museau brun est dessous. Mon ours ! L'ours était sous la poule. Une tasse en bois l'avait caché. Nina le serre contre sa joue. Le poil est chaud, un peu écrasé. Merci d'avoir regardé, Nina. Il buvait en dessous. Te voilà, petit ours. La dernière tasse va dans la caisse. Le tapis a un rond vide, au milieu. Nina pose l'ours contre son genou. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1643,7 +1661,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1651,10 +1669,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1677,30 +1695,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>caisse</t>
+          <t>lune d'étain</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1709,10 +1727,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1725,27 +1743,47 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_la_réussite; emotion=fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_suit_la_lune_trouve_l_ours; tempo=naturel; sourire=franc; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|La deuxième tasse va dans la caisse.
+          <t>enfant-f|J'arrête de pousser.
+narrateur|Elle lâche le tas.
+narrateur|Près de la fenêtre, la lune d'étain brille.
+enfant-f|Elle me montre le tapis.
+narrateur|Nina prend une tasse en bois.
+narrateur|Elle la pose dans la caisse ronde.
 narrateur|Clic.
-narrateur|Nina prend le lapin tout doux.
-narrateur|Elle le glisse dans la caisse.
-maman|Tu regardes bien sous les peluches ?
+papa|La tasse a sa place.
+narrateur|La deuxième tasse suit.
+enfant-f|Toi aussi, lapin.
+narrateur|Elle glisse le lapin dans la caisse.
+maman|Tu regardes bien dessous ?
 enfant-f|Oui, maman.
-narrateur|La poule est encore au milieu.
-papa|Un coin de tapis reparaît.
-narrateur|Nina soulève la poule.
+narrateur|Un coin de tapis reparaît.
+narrateur|La poule reste au milieu.
+enfant-f|Je prends tout d'un coup.
+narrateur|Nina ouvre les deux mains.
+narrateur|Elle veut vider le tapis vite.
+narrateur|La poule bascule sur le côté.
+narrateur|Puis la dernière tasse part sous la chaise.
+enfant-f|Oh non.
+narrateur|Nina s'arrête net.
+enfant-f|Pas comme ça.
+narrateur|Elle refuse de foncer.
+narrateur|Elle lève les yeux vers la boîte.
+narrateur|La lune d'étain capte la pluie.
+narrateur|Un reflet tombe sur un petit dos.
+enfant-f|Là, sous la poule.
+narrateur|Nina soulève la poule, sans se presser.
 narrateur|Un museau brun est dessous.
 enfant-f|Mon ours !
 narrateur|L'ours était sous la poule.
 narrateur|Une tasse en bois l'avait caché.
 narrateur|Nina le serre contre sa joue.
 narrateur|Le poil est chaud, un peu écrasé.
-papa|Merci, tu l'as trouvé.
+papa|Merci d'avoir regardé, Nina.
 enfant-f|Il buvait en dessous.
 maman|Te voilà, petit ours.
 narrateur|La dernière tasse va dans la caisse.
@@ -1753,6 +1791,11 @@
 narrateur|Nina pose l'ours contre son genou.</t>
         </is>
       </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>tasse-bois,caisse</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1777,17 +1820,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Maman pose la vraie tasse au milieu. La vapeur sent le cacao. Il est chaud. On souffle un peu. Nina souffle. Ffff. Elle boit une petite gorgée. Le cacao est doux, un peu sucré. L'ours a une goutte, papa. Une toute petite goutte. Tu veux encore un peu ? Oui, maman. La pluie tapote plus doucement. La chaussette sur la chaise est sèche. Nina tient l'ours d'une main. De l'autre, elle tient la tasse. On est bien, ici.</t>
+          <t>Maman avance la vraie tasse. La vapeur sent le cacao. Je la prends maintenant ! Nina tend les deux mains trop vite. La tasse penche, la vapeur fuit. Elle est chaude, tu vois ? J'attends. Nina pose les mains à plat. Elle souffle une fois, puis deux. Ffff. La lune d'étain éclaire un rond. Là, au milieu. Maman pose la tasse sur ce rond. On souffle un peu. Nina souffle avec lui. Elle boit une petite gorgée. Le cacao est doux, un peu sucré. L'ours a une goutte, papa. Une toute petite goutte. Tu en veux un peu ? Oui, maman.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Maman pose la vraie tasse au milieu. La vapeur sent le cacao. Il est chaud. On souffle un peu. Nina souffle. Ffff. Elle boit une petite gorgée. Le cacao est doux, un peu sucré. L'ours a une goutte, papa. Une toute petite goutte. Tu veux encore un peu ? Oui, maman. La pluie tapote plus doucement. La chaussette sur la chaise est sèche. Nina tient l'ours d'une main. De l'autre, elle tient la tasse. On est bien, ici.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Maman avance la vraie tasse. La vapeur sent le cacao. Je la prends maintenant ! Nina tend les deux mains trop vite. La tasse penche, la vapeur fuit. Elle est chaude, tu vois ? J'attends. Nina pose les mains à plat. Elle souffle une fois, puis deux. Ffff. La &lt;emphasis level="moderate"&gt;lune d'étain&lt;/emphasis&gt; éclaire un rond. Là, au milieu. Maman pose la tasse sur ce rond. On souffle un peu. Nina souffle avec lui. Elle boit une petite gorgée. Le cacao est doux, un peu sucré. L'ours a une goutte, papa. Une toute petite goutte. Tu en veux un peu ? Oui, maman.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Sami ferme la &lt;emphasis&gt;caisse&lt;/emphasis&gt;. Maman lui tend l'eau. [pause]</t>
+          <t>&lt;low-pitch&gt;Maman avance la vraie tasse. La vapeur sent le cacao. Je la prends maintenant ! Nina tend les deux mains trop vite. La tasse penche, la vapeur fuit. Elle est chaude, tu vois ? J'attends. Nina pose les mains à plat. Elle souffle une fois, puis deux. Ffff. La &lt;emphasis&gt;lune d'étain&lt;/emphasis&gt; éclaire un rond. Là, au milieu. Maman pose la tasse sur ce rond. On souffle un peu. Nina souffle avec lui. Elle boit une petite gorgée. Le cacao est doux, un peu sucré. L'ours a une goutte, papa. Une toute petite goutte. Tu en veux un peu ? Oui, maman.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1834,7 +1877,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1842,22 +1885,26 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1868,30 +1915,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>caisse</t>
+          <t>lune d'étain</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1900,40 +1947,53 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=deux_envies_qui_se_heurtent; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_pose_la_tasse; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Maman pose la vraie tasse au milieu.
+          <t>narrateur|Maman avance la vraie tasse.
 narrateur|La vapeur sent le cacao.
-enfant-f|Il est chaud.
+enfant-f|Je la prends maintenant !
+narrateur|Nina tend les deux mains trop vite.
+narrateur|La tasse penche, la vapeur fuit.
+maman|Elle est chaude, tu vois ?
+enfant-f|J'attends.
+narrateur|Nina pose les mains à plat.
+narrateur|Elle souffle une fois, puis deux.
+enfant-f|Ffff.
+narrateur|La lune d'étain éclaire un rond.
+enfant-f|Là, au milieu.
+narrateur|Maman pose la tasse sur ce rond.
 papa|On souffle un peu.
-narrateur|Nina souffle.
-narrateur|Ffff.
+narrateur|Nina souffle avec lui.
 narrateur|Elle boit une petite gorgée.
 narrateur|Le cacao est doux, un peu sucré.
 enfant-f|L'ours a une goutte, papa.
 papa|Une toute petite goutte.
-maman|Tu veux encore un peu ?
-enfant-f|Oui, maman.
-narrateur|La pluie tapote plus doucement.
-narrateur|La chaussette sur la chaise est sèche.
-narrateur|Nina tient l'ours d'une main.
-narrateur|De l'autre, elle tient la tasse.
-maman|On est bien, ici.</t>
+maman|Tu en veux un peu ?
+enfant-f|Oui, maman.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>cacao</t>
         </is>
       </c>
     </row>
@@ -1960,17 +2020,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>L'ours a bu du cacao. Toi aussi. Bravo, tu l'as retrouvé. La vapeur s'en va tout doux. Le tapis reste chaud sous les genoux.</t>
+          <t>La pluie tapote plus bas. La chaussette sur la chaise est sèche. Nina tient l'ours d'une main. De l'autre, elle tient la tasse. La boîte à musique reprend un ding. On est bien, ici. Oui, vous y êtes. La vapeur s'accroche à la lune d'étain.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>L'ours a bu du cacao. Toi aussi. Bravo, tu l'as retrouvé. La vapeur s'en va tout doux. Le tapis reste chaud sous les genoux.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La pluie tapote plus bas. La chaussette sur la chaise est sèche. Nina tient l'ours d'une main. De l'autre, elle tient la tasse. La boîte à musique reprend un ding. On est bien, ici. Oui, vous y êtes. La vapeur s'accroche à la &lt;emphasis level="moderate"&gt;lune d'étain&lt;/emphasis&gt;.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La pluie tapote plus bas. La chaussette sur la chaise est sèche. Nina tient l'ours d'une main. De l'autre, elle tient la tasse. La boîte à musique reprend un ding. On est bien, ici. Oui, vous y êtes. La vapeur s'accroche à la &lt;emphasis&gt;lune d'étain&lt;/emphasis&gt;.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2017,18 +2077,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2037,12 +2097,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2051,17 +2111,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>lune d'étain</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2070,11 +2134,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2083,28 +2147,40 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=la_vapeur_s_accroche_a_la_lune_detain; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|L'ours a bu du cacao.
-maman|Toi aussi.
-papa|Bravo, tu l'as retrouvé.
-narrateur|La vapeur s'en va tout doux.
-narrateur|Le tapis reste chaud sous les genoux.</t>
+          <t>narrateur|La pluie tapote plus bas.
+narrateur|La chaussette sur la chaise est sèche.
+narrateur|Nina tient l'ours d'une main.
+narrateur|De l'autre, elle tient la tasse.
+narrateur|La boîte à musique reprend un ding.
+enfant-f|On est bien, ici.
+maman|Oui, vous y êtes.
+narrateur|La vapeur s'accroche à la lune d'étain.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>pluie,boite-musique</t>
         </is>
       </c>
     </row>
@@ -2125,7 +2201,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2189,6 +2265,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>